<commit_message>
Week 2 results, week 3 picks
</commit_message>
<xml_diff>
--- a/picks/RoachFinder_Picks_2026-27.xlsx
+++ b/picks/RoachFinder_Picks_2026-27.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Week 02" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Week 03" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -547,7 +548,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -594,7 +594,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -641,7 +640,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -688,7 +686,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -735,7 +732,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -772,13 +768,11 @@
       <c r="H7" t="n">
         <v>3.75</v>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -815,13 +809,11 @@
       <c r="H8" t="n">
         <v>2.82</v>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -858,13 +850,11 @@
       <c r="H9" t="n">
         <v>2.75</v>
       </c>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -901,6 +891,744 @@
       <c r="H10" t="n">
         <v>2.64</v>
       </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Minnesota Vikings</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Chicago Bears</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>CHI -4.5</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Vikings +4.5</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>1.67</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>4:25 PM</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Seattle Seahawks</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Arizona Cardinals</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SEA -3.5</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Cardinals +3.5</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>1.43</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>New Orleans Saints</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Baltimore Ravens</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>BAL -8.5</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Saints +8.5</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>8:15 PM</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>New York Giants</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Los Angeles Rams</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LAR -7</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Giants +7.0</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Cincinnati Bengals</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Houston Texans</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>HOU -3</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Texans -3.0</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>1.14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Pittsburgh Steelers</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>New England Patriots</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>NE -5.5</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Steelers +5.5</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Philadelphia Eagles</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Tennessee Titans</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PHI -7</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Titans +7.0</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Rolling median CF:</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2.695</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Game Time</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Vegas Line</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>O/U</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Pick</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Top 5</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Above Median</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Result (W/L/P)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>8:15 PM</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Philadelphia Eagles</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Chicago Bears</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PHI -3.5</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Bears +3.5</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>8.539999999999999</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Houston Texans</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Indianapolis Colts</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>HOU -2.5</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Colts +2.5</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>New York Jets</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Detroit Lions</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>DET -6.5</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Jets +6.5</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>8:15 PM</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Atlanta Falcons</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Green Bay Packers</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>GB -6</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Falcons +6.0</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>4:25 PM</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Baltimore Ravens</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Dallas Cowboys</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>BAL -3</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Cowboys +3.0</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Seattle Seahawks</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Washington Commanders</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SEA -7</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Commanders +7.0</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Los Angeles Chargers</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Buffalo Bills</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BUF -7</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Bills -7.0</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Cincinnati Bengals</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Pittsburgh Steelers</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>CIN -3.5</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Steelers +3.5</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>4:25 PM</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Las Vegas Raiders</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>New Orleans Saints</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>NO -3</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Raiders +3.0</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>1.1</v>
+      </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -916,29 +1644,29 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Minnesota Vikings</t>
+          <t>Carolina Panthers</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Chicago Bears</t>
+          <t>Cleveland Browns</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CHI -4.5</t>
+          <t>CAR -2.5</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>47.5</v>
+        <v>42.5</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Vikings +4.5</t>
+          <t>Browns +2.5</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>1.67</v>
+        <v>1.05</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -950,34 +1678,34 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4:25 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Seattle Seahawks</t>
+          <t>Kansas City Chiefs</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Arizona Cardinals</t>
+          <t>Miami Dolphins</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEA -3.5</t>
+          <t>KC -11.5</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>41.5</v>
+        <v>45.5</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Cardinals +3.5</t>
+          <t>Dolphins +11.5</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1.43</v>
+        <v>1.04</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -989,34 +1717,34 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>4:05 PM</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>New Orleans Saints</t>
+          <t>Minnesota Vikings</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Baltimore Ravens</t>
+          <t>Tampa Bay Buccaneers</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BAL -8.5</t>
+          <t>MIN -1.5</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>46.5</v>
+        <v>42.5</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Saints +8.5</t>
+          <t>Vikings -1.5</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1.35</v>
+        <v>0.93</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -1028,34 +1756,34 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>8:15 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>New York Giants</t>
+          <t>New England Patriots</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Los Angeles Rams</t>
+          <t>Jacksonville Jaguars</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>LAR -7</t>
+          <t>JAX -3</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>47.5</v>
+        <v>45.5</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Giants +7.0</t>
+          <t>Patriots +3.0</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1.3</v>
+        <v>0.74</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -1067,34 +1795,34 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>4:05 PM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Cincinnati Bengals</t>
+          <t>Arizona Cardinals</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Houston Texans</t>
+          <t>San Francisco 49ers</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>HOU -3</t>
+          <t>SF -8.5</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>46.5</v>
+        <v>47.5</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Texans -3.0</t>
+          <t>49ers -8.5</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1.14</v>
+        <v>0.73</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
@@ -1106,34 +1834,34 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>8:20 PM</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Pittsburgh Steelers</t>
+          <t>Los Angeles Rams</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>New England Patriots</t>
+          <t>Denver Broncos</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>NE -5.5</t>
+          <t>LAR -2.5</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>41.5</v>
+        <v>45.5</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Steelers +5.5</t>
+          <t>Rams -2.5</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>0.84</v>
+        <v>0.46</v>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
@@ -1150,29 +1878,29 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Philadelphia Eagles</t>
+          <t>Tennessee Titans</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Tennessee Titans</t>
+          <t>New York Giants</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>PHI -7</t>
+          <t>NYG -3.5</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>39.5</v>
+        <v>40.5</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Titans +7.0</t>
+          <t>Giants -3.5</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
@@ -1185,7 +1913,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>2.695</v>
+        <v>1.65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Week 3 results, week 4 picks
</commit_message>
<xml_diff>
--- a/picks/RoachFinder_Picks_2026-27.xlsx
+++ b/picks/RoachFinder_Picks_2026-27.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Week 02" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Week 03" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Week 04" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1283,7 +1284,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1330,7 +1330,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1377,7 +1376,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1424,7 +1422,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1471,7 +1468,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1508,13 +1504,11 @@
       <c r="H7" t="n">
         <v>1.76</v>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1551,9 +1545,6 @@
       <c r="H8" t="n">
         <v>1.63</v>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1590,9 +1581,6 @@
       <c r="H9" t="n">
         <v>1.3</v>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1629,9 +1617,6 @@
       <c r="H10" t="n">
         <v>1.1</v>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1668,9 +1653,6 @@
       <c r="H11" t="n">
         <v>1.05</v>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1707,6 +1689,766 @@
       <c r="H12" t="n">
         <v>1.04</v>
       </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>4:05 PM</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Minnesota Vikings</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Tampa Bay Buccaneers</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>MIN -1.5</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Vikings -1.5</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>New England Patriots</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Jacksonville Jaguars</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>JAX -3</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Patriots +3.0</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>0.74</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>4:05 PM</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Arizona Cardinals</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>San Francisco 49ers</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>SF -8.5</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>49ers -8.5</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>8:20 PM</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Los Angeles Rams</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Denver Broncos</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LAR -2.5</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Rams -2.5</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Tennessee Titans</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>New York Giants</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>NYG -3.5</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Giants -3.5</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Rolling median CF:</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1.65</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Game Time</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Vegas Line</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>O/U</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Pick</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Top 5</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Above Median</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Result (W/L/P)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>9:30 AM</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Indianapolis Colts</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Washington Commanders</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>IND -3.5</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Commanders +3.5</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>7.67</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>8:15 PM</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Pittsburgh Steelers</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Cleveland Browns</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PIT -2.5</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Browns +2.5</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>5.58</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>New York Jets</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Chicago Bears</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>CHI -3.5</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Bears -3.5</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4:25 PM</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Denver Broncos</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>San Francisco 49ers</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SF -3</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>49ers -3.0</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Green Bay Packers</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Tampa Bay Buccaneers</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>GB -3.5</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Buccaneers +3.5</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Jacksonville Jaguars</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Cincinnati Bengals</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>CIN -2.5</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Jaguars +2.5</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>4:25 PM</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Los Angeles Chargers</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Seattle Seahawks</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>SEA -7</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Seahawks -7.0</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8:15 PM</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Atlanta Falcons</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>New Orleans Saints</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>NO -3</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Falcons +3.0</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Tennessee Titans</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Baltimore Ravens</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>BAL -11.5</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Titans +11.5</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Los Angeles Rams</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Philadelphia Eagles</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LAR -3</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Rams -3.0</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>New England Patriots</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Buffalo Bills</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>BUF -7</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Patriots +7.0</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>2.33</v>
+      </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -1717,34 +2459,34 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>4:05 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Minnesota Vikings</t>
+          <t>Arizona Cardinals</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Tampa Bay Buccaneers</t>
+          <t>New York Giants</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MIN -1.5</t>
+          <t>ARI -1.5</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>42.5</v>
+        <v>44.5</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Vikings -1.5</t>
+          <t>Giants +1.5</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0.93</v>
+        <v>1.79</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -1756,34 +2498,34 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>8:20 PM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>New England Patriots</t>
+          <t>Detroit Lions</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Jacksonville Jaguars</t>
+          <t>Carolina Panthers</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>JAX -3</t>
+          <t>DET -3.5</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>45.5</v>
+        <v>50.5</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Patriots +3.0</t>
+          <t>Panthers +3.5</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0.74</v>
+        <v>1.57</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -1795,22 +2537,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>4:05 PM</t>
+          <t>4:25 PM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Arizona Cardinals</t>
+          <t>Kansas City Chiefs</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>San Francisco 49ers</t>
+          <t>Las Vegas Raiders</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SF -8.5</t>
+          <t>KC -4.5</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1818,11 +2560,11 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>49ers -8.5</t>
+          <t>Raiders +4.5</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>0.73</v>
+        <v>1.45</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
@@ -1834,34 +2576,34 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>8:20 PM</t>
+          <t>4:05 PM</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Los Angeles Rams</t>
+          <t>Miami Dolphins</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Denver Broncos</t>
+          <t>Minnesota Vikings</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>LAR -2.5</t>
+          <t>MIN -11.5</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>45.5</v>
+        <v>38.5</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Rams -2.5</t>
+          <t>Vikings -11.5</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>0.46</v>
+        <v>1.22</v>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
@@ -1878,29 +2620,29 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tennessee Titans</t>
+          <t>Dallas Cowboys</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>New York Giants</t>
+          <t>Houston Texans</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>NYG -3.5</t>
+          <t>HOU -2.5</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>40.5</v>
+        <v>47.5</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Giants -3.5</t>
+          <t>Cowboys +2.5</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>0.16</v>
+        <v>0.22</v>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
@@ -1913,7 +2655,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1.65</v>
+        <v>2.335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Week 4 results, week 5 picks
</commit_message>
<xml_diff>
--- a/picks/RoachFinder_Picks_2026-27.xlsx
+++ b/picks/RoachFinder_Picks_2026-27.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Week 02" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Week 03" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Week 04" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Week 05" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2009,7 +2010,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -2056,7 +2056,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -2103,7 +2102,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -2150,7 +2148,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -2197,7 +2194,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2234,13 +2230,11 @@
       <c r="H7" t="n">
         <v>3.44</v>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2277,13 +2271,11 @@
       <c r="H8" t="n">
         <v>2.98</v>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -2320,13 +2312,11 @@
       <c r="H9" t="n">
         <v>2.81</v>
       </c>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -2363,13 +2353,11 @@
       <c r="H10" t="n">
         <v>2.53</v>
       </c>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -2406,13 +2394,11 @@
       <c r="H11" t="n">
         <v>2.47</v>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2449,6 +2435,758 @@
       <c r="H12" t="n">
         <v>2.33</v>
       </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Arizona Cardinals</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>New York Giants</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ARI -1.5</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Giants +1.5</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>1.79</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>8:20 PM</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Detroit Lions</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Carolina Panthers</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>DET -3.5</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Panthers +3.5</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>1.57</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>4:25 PM</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Kansas City Chiefs</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Las Vegas Raiders</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>KC -4.5</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Raiders +4.5</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>1.45</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>4:05 PM</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Miami Dolphins</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Minnesota Vikings</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>MIN -11.5</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Vikings -11.5</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>1.22</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Dallas Cowboys</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Houston Texans</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>HOU -2.5</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Cowboys +2.5</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Rolling median CF:</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2.335</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Game Time</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Vegas Line</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>O/U</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Pick</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Top 5</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Above Median</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Result (W/L/P)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>9:30 AM</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Philadelphia Eagles</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Jacksonville Jaguars</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>JAX -6.5</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Jaguars -6.5</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Indianapolis Colts</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Pittsburgh Steelers</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PIT -2.5</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Colts +2.5</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Houston Texans</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Tennessee Titans</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>HOU -6.5</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Titans +6.5</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4:25 PM</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Detroit Lions</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Arizona Cardinals</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DET -4.5</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Cardinals +4.5</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>8:15 PM</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Buffalo Bills</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Los Angeles Rams</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LAR -2.5</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Rams -2.5</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Minnesota Vikings</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>New Orleans Saints</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>MIN -1.5</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Vikings -1.5</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>8:15 PM</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Tampa Bay Buccaneers</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Dallas Cowboys</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>DAL -8.5</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Buccaneers +8.5</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>4:05 PM</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Denver Broncos</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Los Angeles Chargers</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>DEN -3.5</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Chargers +3.5</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Chicago Bears</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Green Bay Packers</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>CHI -3</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Bears -3.0</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Cleveland Browns</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>New York Jets</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>NYJ -2.5</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Browns +2.5</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>4:25 PM</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>San Francisco 49ers</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Seattle Seahawks</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SEA -3</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>49ers +3.0</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>1.86</v>
+      </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -2464,29 +3202,29 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Arizona Cardinals</t>
+          <t>Cincinnati Bengals</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>New York Giants</t>
+          <t>Miami Dolphins</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ARI -1.5</t>
+          <t>CIN -7</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>44.5</v>
+        <v>42.5</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Giants +1.5</t>
+          <t>Dolphins +7.0</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1.79</v>
+        <v>1.24</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -2503,29 +3241,29 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Detroit Lions</t>
+          <t>Baltimore Ravens</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Carolina Panthers</t>
+          <t>Atlanta Falcons</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>DET -3.5</t>
+          <t>ATL -3</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>50.5</v>
+        <v>43.5</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Panthers +3.5</t>
+          <t>Ravens +3.0</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1.57</v>
+        <v>1.1</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -2537,34 +3275,34 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>4:25 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Kansas City Chiefs</t>
+          <t>Las Vegas Raiders</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Las Vegas Raiders</t>
+          <t>New England Patriots</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>KC -4.5</t>
+          <t>NE -3.5</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>47.5</v>
+        <v>45.5</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Raiders +4.5</t>
+          <t>Raiders +3.5</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1.45</v>
+        <v>1.06</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
@@ -2576,86 +3314,47 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>4:05 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Miami Dolphins</t>
+          <t>New York Giants</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Minnesota Vikings</t>
+          <t>Washington Commanders</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>MIN -11.5</t>
+          <t>WSH -3.5</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>38.5</v>
+        <v>43.5</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Vikings -11.5</t>
+          <t>Giants +3.5</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>1.22</v>
+        <v>0.73</v>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
     </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>1:00 PM</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Dallas Cowboys</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Houston Texans</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>HOU -2.5</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Cowboys +2.5</t>
-        </is>
-      </c>
-      <c r="H17" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Rolling median CF:</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>2.335</v>
+      <c r="D18" t="n">
+        <v>2.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Week 5 results, week 6 picks
</commit_message>
<xml_diff>
--- a/picks/RoachFinder_Picks_2026-27.xlsx
+++ b/picks/RoachFinder_Picks_2026-27.xlsx
@@ -2729,21 +2729,15 @@
           <t>Jacksonville Jaguars</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>JAX -6.5</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>42.5</v>
-      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Jaguars -6.5</t>
+          <t>Jaguars (no line)</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>5.2</v>
+        <v>11.7</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -2763,34 +2757,28 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>8:15 PM</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Indianapolis Colts</t>
+          <t>Tampa Bay Buccaneers</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Pittsburgh Steelers</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>PIT -2.5</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>44.5</v>
-      </c>
+          <t>Dallas Cowboys</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Colts +2.5</t>
+          <t>Cowboys (no line)</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>4.53</v>
+        <v>5.97</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -2810,34 +2798,28 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>8:15 PM</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Houston Texans</t>
+          <t>Buffalo Bills</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Tennessee Titans</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>HOU -6.5</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>38.5</v>
-      </c>
+          <t>Los Angeles Rams</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Titans +6.5</t>
+          <t>Rams (no line)</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>4.21</v>
+        <v>5.95</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -2857,34 +2839,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4:25 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Detroit Lions</t>
+          <t>Cincinnati Bengals</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Arizona Cardinals</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>DET -4.5</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>54.5</v>
-      </c>
+          <t>Miami Dolphins</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Cardinals +4.5</t>
+          <t>Bengals (no line)</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>4.04</v>
+        <v>5.76</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -2904,34 +2880,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>8:15 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Buffalo Bills</t>
+          <t>Chicago Bears</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Los Angeles Rams</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>LAR -2.5</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>54.5</v>
-      </c>
+          <t>Green Bay Packers</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Rams -2.5</t>
+          <t>Bears (no line)</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>3.45</v>
+        <v>5.21</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -2964,21 +2934,15 @@
           <t>New Orleans Saints</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>MIN -1.5</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>42.5</v>
-      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Vikings -1.5</t>
+          <t>Vikings (no line)</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>3.31</v>
+        <v>4.81</v>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
@@ -2994,34 +2958,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8:15 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tampa Bay Buccaneers</t>
+          <t>New York Giants</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Dallas Cowboys</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>DAL -8.5</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>47.5</v>
-      </c>
+          <t>Washington Commanders</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Buccaneers +8.5</t>
+          <t>Commanders (no line)</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>2.53</v>
+        <v>2.77</v>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
@@ -3037,34 +2995,28 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>4:05 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Denver Broncos</t>
+          <t>Las Vegas Raiders</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Los Angeles Chargers</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>DEN -3.5</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>42.5</v>
-      </c>
+          <t>New England Patriots</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Chargers +3.5</t>
+          <t>Patriots (no line)</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>2.41</v>
+        <v>2.44</v>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
@@ -3085,29 +3037,23 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Chicago Bears</t>
+          <t>Houston Texans</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Green Bay Packers</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>CHI -3</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>45.5</v>
-      </c>
+          <t>Tennessee Titans</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Bears -3.0</t>
+          <t>Texans (no line)</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>2.21</v>
+        <v>2.29</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -3124,29 +3070,23 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Cleveland Browns</t>
+          <t>Indianapolis Colts</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>New York Jets</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>NYJ -2.5</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>39.5</v>
-      </c>
+          <t>Pittsburgh Steelers</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Browns +2.5</t>
+          <t>Colts (no line)</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>2.21</v>
+        <v>2.03</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -3158,34 +3098,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4:25 PM</t>
+          <t>8:20 PM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>San Francisco 49ers</t>
+          <t>Baltimore Ravens</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Seattle Seahawks</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>SEA -3</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>47.5</v>
-      </c>
+          <t>Atlanta Falcons</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>49ers +3.0</t>
+          <t>Falcons (no line)</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1.86</v>
+        <v>1.9</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -3197,34 +3131,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>4:25 PM</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Cincinnati Bengals</t>
+          <t>San Francisco 49ers</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Miami Dolphins</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>CIN -7</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>42.5</v>
-      </c>
+          <t>Seattle Seahawks</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Dolphins +7.0</t>
+          <t>Seahawks (no line)</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1.24</v>
+        <v>1.14</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -3236,34 +3164,28 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>8:20 PM</t>
+          <t>4:05 PM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Baltimore Ravens</t>
+          <t>Denver Broncos</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Atlanta Falcons</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>ATL -3</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>43.5</v>
-      </c>
+          <t>Los Angeles Chargers</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Ravens +3.0</t>
+          <t>Broncos (no line)</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -3275,34 +3197,28 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>4:25 PM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Las Vegas Raiders</t>
+          <t>Detroit Lions</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>New England Patriots</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>NE -3.5</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
-        <v>45.5</v>
-      </c>
+          <t>Arizona Cardinals</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Raiders +3.5</t>
+          <t>Lions (no line)</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1.06</v>
+        <v>0.46</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
@@ -3319,29 +3235,23 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>New York Giants</t>
+          <t>Cleveland Browns</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Washington Commanders</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>WSH -3.5</t>
-        </is>
-      </c>
-      <c r="F16" t="n">
-        <v>43.5</v>
-      </c>
+          <t>New York Jets</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Giants +3.5</t>
+          <t>Jets (no line)</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>0.73</v>
+        <v>0.29</v>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
@@ -3354,7 +3264,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2.34</v>
+        <v>2.375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Week 6 results posted, backfill created, week 7 picks
</commit_message>
<xml_diff>
--- a/picks/RoachFinder_Picks_2026-27.xlsx
+++ b/picks/RoachFinder_Picks_2026-27.xlsx
@@ -11,6 +11,8 @@
     <sheet name="Week 03" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Week 04" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Week 05" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Week 06" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Week 07" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2729,8 +2731,6 @@
           <t>Jacksonville Jaguars</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Jaguars (no line)</t>
@@ -2749,7 +2749,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -2770,8 +2769,6 @@
           <t>Dallas Cowboys</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>Cowboys (no line)</t>
@@ -2790,7 +2787,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -2811,8 +2807,6 @@
           <t>Los Angeles Rams</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>Rams (no line)</t>
@@ -2831,7 +2825,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -2852,8 +2845,6 @@
           <t>Miami Dolphins</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Bengals (no line)</t>
@@ -2872,7 +2863,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -2893,8 +2883,6 @@
           <t>Green Bay Packers</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>Bears (no line)</t>
@@ -2913,7 +2901,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2934,8 +2921,6 @@
           <t>New Orleans Saints</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>Vikings (no line)</t>
@@ -2944,13 +2929,11 @@
       <c r="H7" t="n">
         <v>4.81</v>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2971,8 +2954,6 @@
           <t>Washington Commanders</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>Commanders (no line)</t>
@@ -2981,13 +2962,11 @@
       <c r="H8" t="n">
         <v>2.77</v>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -3008,8 +2987,6 @@
           <t>New England Patriots</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>Patriots (no line)</t>
@@ -3018,13 +2995,11 @@
       <c r="H9" t="n">
         <v>2.44</v>
       </c>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -3045,8 +3020,6 @@
           <t>Tennessee Titans</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>Texans (no line)</t>
@@ -3054,6 +3027,1322 @@
       </c>
       <c r="H10" t="n">
         <v>2.29</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Indianapolis Colts</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Pittsburgh Steelers</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Colts (no line)</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>2.03</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>8:20 PM</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Baltimore Ravens</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Atlanta Falcons</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Falcons (no line)</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>4:25 PM</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>San Francisco 49ers</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Seattle Seahawks</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Seahawks (no line)</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>1.14</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>4:05 PM</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Denver Broncos</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Los Angeles Chargers</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Broncos (no line)</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>1.09</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>4:25 PM</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Detroit Lions</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Arizona Cardinals</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Lions (no line)</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Cleveland Browns</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>New York Jets</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Jets (no line)</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Rolling median CF:</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2.375</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Game Time</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Vegas Line</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>O/U</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Pick</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Top 5</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Above Median</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Result (W/L/P)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>8:20 PM</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Dallas Cowboys</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Green Bay Packers</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>DAL -1.5</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Packers +1.5</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>6.17</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>New Orleans Saints</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>New York Giants</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NO -1.5</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Giants +1.5</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>4:25 PM</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Los Angeles Chargers</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Kansas City Chiefs</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>KC -7.5</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Chiefs -7.5</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>8:15 PM</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Seattle Seahawks</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Denver Broncos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SEA -3</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Broncos +3.0</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Chicago Bears</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Atlanta Falcons</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>CHI -1.5</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Falcons +1.5</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Tennessee Titans</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Indianapolis Colts</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>IND -6.5</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Colts -6.5</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>New York Jets</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>New England Patriots</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>NE -7.5</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Jets +7.5</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>9:30 AM</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Houston Texans</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Jacksonville Jaguars</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>JAX -2.5</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Jaguars -2.5</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>8:15 PM</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Washington Commanders</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>San Francisco 49ers</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SF -7.5</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>49ers -7.5</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>2.17</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Pittsburgh Steelers</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Tampa Bay Buccaneers</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>PIT -2.5</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Buccaneers +2.5</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>2.08</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>4:05 PM</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Arizona Cardinals</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Los Angeles Rams</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LAR -13.5</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Cardinals +13.5</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>2.08</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>4:25 PM</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Buffalo Bills</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Las Vegas Raiders</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>BUF -5.5</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Raiders +5.5</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>1.85</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Carolina Panthers</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Philadelphia Eagles</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>CAR -3</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Eagles +3.0</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Baltimore Ravens</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Cleveland Browns</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>BAL -3</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Browns +3.0</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Rolling median CF:</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2.34</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Game Time</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Vegas Line</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>O/U</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Pick</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Top 5</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Above Median</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Result (W/L/P)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>8:20 PM</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Kansas City Chiefs</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Seattle Seahawks</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SEA -3</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Chiefs +3.0</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>9:30 AM</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Pittsburgh Steelers</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>New Orleans Saints</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PIT -3.5</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Saints +3.5</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>San Francisco 49ers</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Atlanta Falcons</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SF -3</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>49ers -3.0</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>New York Giants</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Houston Texans</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>HOU -10</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Giants +10.0</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Miami Dolphins</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>New York Jets</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>NYJ -4.5</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Jets -4.5</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>8:15 PM</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Dallas Cowboys</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Philadelphia Eagles</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>DAL -4.5</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Eagles +4.5</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>8:15 PM</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>New England Patriots</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Chicago Bears</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>CHI -3</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Patriots +3.0</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>4:05 PM</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Denver Broncos</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Arizona Cardinals</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>DEN -4.5</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Cardinals +4.5</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Tampa Bay Buccaneers</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Carolina Panthers</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>CAR -3.5</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Panthers -3.5</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>1.42</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -3075,18 +4364,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Pittsburgh Steelers</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+          <t>Minnesota Vikings</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>MIN -6.5</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>41.5</v>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Colts (no line)</t>
+          <t>Vikings -6.5</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>2.03</v>
+        <v>1.33</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -3098,28 +4393,34 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>8:20 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Baltimore Ravens</t>
+          <t>Cleveland Browns</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Atlanta Falcons</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+          <t>Tennessee Titans</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CLE -1.5</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>37.5</v>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Falcons (no line)</t>
+          <t>Browns -1.5</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1.9</v>
+        <v>0.83</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -3131,28 +4432,34 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>4:25 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>San Francisco 49ers</t>
+          <t>Cincinnati Bengals</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Seattle Seahawks</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
+          <t>Baltimore Ravens</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>BAL -3</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>51.5</v>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Seahawks (no line)</t>
+          <t>Ravens -3.0</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1.14</v>
+        <v>0.52</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -3164,28 +4471,34 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>4:05 PM</t>
+          <t>4:25 PM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Denver Broncos</t>
+          <t>Los Angeles Rams</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Los Angeles Chargers</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
+          <t>Las Vegas Raiders</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LAR -4.5</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>48.5</v>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Broncos (no line)</t>
+          <t>Raiders +4.5</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1.09</v>
+        <v>0.37</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -3202,69 +4515,42 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>Green Bay Packers</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>Detroit Lions</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Arizona Cardinals</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>DET -3</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>53.5</v>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Lions (no line)</t>
+          <t>Lions -3.0</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>0.46</v>
+        <v>0.04</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
     </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>1:00 PM</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Cleveland Browns</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>New York Jets</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Jets (no line)</t>
-        </is>
-      </c>
-      <c r="H16" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Rolling median CF:</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>2.375</v>
+      <c r="D17" t="n">
+        <v>2.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>